<commit_message>
vault backup: 2026-09-28 17:46:54
</commit_message>
<xml_diff>
--- a/ПРЕДМЕТЫ/Математические методы и модели поддержки принятия решений/Лабораторные работы/Лист Microsoft Excel.xlsx
+++ b/ПРЕДМЕТЫ/Математические методы и модели поддержки принятия решений/Лабораторные работы/Лист Microsoft Excel.xlsx
@@ -1,31 +1,133 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\obsidian-dvfu_p2\ПРЕДМЕТЫ\Математические методы и модели поддержки принятия решений\Лабораторные работы\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65D0F89A-E271-4D73-BABE-EF1C3595B074}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Лист1" sheetId="1" r:id="rId1"/>
+    <sheet name="Лист2" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <definedNames>
+    <definedName name="solver_adj" localSheetId="0" hidden="1">Лист2!$C$3:$C$4</definedName>
+    <definedName name="solver_cvg" localSheetId="0" hidden="1">0.0001</definedName>
+    <definedName name="solver_drv" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_eng" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_est" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_itr" localSheetId="0" hidden="1">2147483647</definedName>
+    <definedName name="solver_lhs1" localSheetId="0" hidden="1">Лист2!$C$10</definedName>
+    <definedName name="solver_lhs2" localSheetId="0" hidden="1">Лист2!$C$11</definedName>
+    <definedName name="solver_lhs3" localSheetId="0" hidden="1">Лист2!$C$12</definedName>
+    <definedName name="solver_lhs4" localSheetId="0" hidden="1">Лист2!$C$13</definedName>
+    <definedName name="solver_lhs5" localSheetId="0" hidden="1">Лист2!$C$9</definedName>
+    <definedName name="solver_lhs6" localSheetId="0" hidden="1">Лист2!$D$9</definedName>
+    <definedName name="solver_mip" localSheetId="0" hidden="1">2147483647</definedName>
+    <definedName name="solver_mni" localSheetId="0" hidden="1">30</definedName>
+    <definedName name="solver_mrt" localSheetId="0" hidden="1">0.075</definedName>
+    <definedName name="solver_msl" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_neg" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_nod" localSheetId="0" hidden="1">2147483647</definedName>
+    <definedName name="solver_num" localSheetId="0" hidden="1">6</definedName>
+    <definedName name="solver_nwt" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_opt" localSheetId="0" hidden="1">Лист2!$C$6</definedName>
+    <definedName name="solver_pre" localSheetId="0" hidden="1">0.000001</definedName>
+    <definedName name="solver_rbv" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_rel1" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_rel2" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_rel3" localSheetId="0" hidden="1">3</definedName>
+    <definedName name="solver_rel4" localSheetId="0" hidden="1">3</definedName>
+    <definedName name="solver_rel5" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_rel6" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_rhs1" localSheetId="0" hidden="1">Лист2!$D$10</definedName>
+    <definedName name="solver_rhs2" localSheetId="0" hidden="1">Лист2!$D$11</definedName>
+    <definedName name="solver_rhs3" localSheetId="0" hidden="1">Лист2!$D$12</definedName>
+    <definedName name="solver_rhs4" localSheetId="0" hidden="1">Лист2!$D$13</definedName>
+    <definedName name="solver_rhs5" localSheetId="0" hidden="1">Лист2!$C$8</definedName>
+    <definedName name="solver_rhs6" localSheetId="0" hidden="1">Лист2!$D$8</definedName>
+    <definedName name="solver_rlx" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_rsd" localSheetId="0" hidden="1">0</definedName>
+    <definedName name="solver_scl" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_sho" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_ssz" localSheetId="0" hidden="1">100</definedName>
+    <definedName name="solver_tim" localSheetId="0" hidden="1">2147483647</definedName>
+    <definedName name="solver_tol" localSheetId="0" hidden="1">0.01</definedName>
+    <definedName name="solver_typ" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_val" localSheetId="0" hidden="1">0</definedName>
+    <definedName name="solver_ver" localSheetId="0" hidden="1">3</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+  <si>
+    <t>ЛИНЕЙНАЯ ОПТИМИЗАЦИЯ ПЛАНИРОВАНИЯ ПРОИЗВОДСТВА МАТЕРИАЛОВ</t>
+  </si>
+  <si>
+    <t>Суточный объем производства материала A</t>
+  </si>
+  <si>
+    <t>Суточный объем производства материала B</t>
+  </si>
+  <si>
+    <t>Целевая функция</t>
+  </si>
+  <si>
+    <t>Ограничения</t>
+  </si>
+  <si>
+    <t>По запасам на складе</t>
+  </si>
+  <si>
+    <t>На величину спроса</t>
+  </si>
+  <si>
+    <t>По знаку</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -49,11 +151,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -330,10 +444,133 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96F59ECD-39EC-4923-B56C-5702F6ADBABD}">
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="2" width="16.33203125" style="2" customWidth="1"/>
+    <col min="3" max="7" width="10.5546875" style="2" customWidth="1"/>
+    <col min="8" max="16384" width="8.88671875" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+    </row>
+    <row r="3" spans="1:7" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1"/>
+      <c r="C3" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1"/>
+      <c r="C4" s="4">
+        <v>1.9999999999999998</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="1"/>
+      <c r="C6" s="4">
+        <f>3000*C3 + 4000*C4</f>
+        <v>11000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="1"/>
+    </row>
+    <row r="8" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="1"/>
+      <c r="C8" s="2">
+        <v>9</v>
+      </c>
+      <c r="D8" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C9" s="2">
+        <f>5*C3 + 2 * C4</f>
+        <v>9</v>
+      </c>
+      <c r="D9" s="2">
+        <f>2*C3 + 4*C4</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B10" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="2">
+        <f>C4-C3</f>
+        <v>0.99999999999999978</v>
+      </c>
+      <c r="D10" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C11" s="2">
+        <f>C3</f>
+        <v>1</v>
+      </c>
+      <c r="D11" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="2">
+        <f>C3</f>
+        <v>1</v>
+      </c>
+      <c r="D12" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C13" s="2">
+        <f>C4</f>
+        <v>1.9999999999999998</v>
+      </c>
+      <c r="D13" s="2">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-09-28 17:48:24
</commit_message>
<xml_diff>
--- a/ПРЕДМЕТЫ/Математические методы и модели поддержки принятия решений/Лабораторные работы/Лист Microsoft Excel.xlsx
+++ b/ПРЕДМЕТЫ/Математические методы и модели поддержки принятия решений/Лабораторные работы/Лист Microsoft Excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\obsidian-dvfu_p2\ПРЕДМЕТЫ\Математические методы и модели поддержки принятия решений\Лабораторные работы\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65D0F89A-E271-4D73-BABE-EF1C3595B074}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE10BE59-642D-45F6-B156-CDC8C3E360A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист2" sheetId="2" r:id="rId1"/>
@@ -151,19 +151,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -448,9 +451,9 @@
   <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="16.33203125" style="2" customWidth="1"/>
-    <col min="3" max="7" width="10.5546875" style="2" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="2"/>
+    <col min="1" max="2" width="16.33203125" style="1" customWidth="1"/>
+    <col min="3" max="7" width="10.5546875" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -465,111 +468,123 @@
       <c r="G1" s="3"/>
     </row>
     <row r="3" spans="1:7" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="4">
+      <c r="B3" s="4"/>
+      <c r="C3" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="1"/>
-      <c r="C4" s="4">
+      <c r="B4" s="4"/>
+      <c r="C4" s="2">
         <v>1.9999999999999998</v>
       </c>
     </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="5"/>
+      <c r="B5" s="5"/>
+    </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="1"/>
-      <c r="C6" s="4">
+      <c r="B6" s="4"/>
+      <c r="C6" s="2">
         <f>3000*C3 + 4000*C4</f>
         <v>11000</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="1"/>
+      <c r="B7" s="4"/>
     </row>
     <row r="8" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="1"/>
-      <c r="C8" s="2">
+      <c r="B8" s="4"/>
+      <c r="C8" s="1">
         <v>9</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="1">
         <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C9" s="2">
+      <c r="A9" s="5"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="1">
         <f>5*C3 + 2 * C4</f>
         <v>9</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="1">
         <f>2*C3 + 4*C4</f>
         <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B10" s="2" t="s">
+      <c r="A10" s="5"/>
+      <c r="B10" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="1">
         <f>C4-C3</f>
         <v>0.99999999999999978</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C11" s="2">
+      <c r="A11" s="5"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="1">
         <f>C3</f>
         <v>1</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11" s="1">
         <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B12" s="2" t="s">
+      <c r="A12" s="5"/>
+      <c r="B12" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="1">
         <f>C3</f>
         <v>1</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C13" s="2">
+      <c r="A13" s="5"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="1">
         <f>C4</f>
         <v>1.9999999999999998</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="A8:B8"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>